<commit_message>
feat(core): add image renderer columns
</commit_message>
<xml_diff>
--- a/packages/core/examples/playground.xlsx
+++ b/packages/core/examples/playground.xlsx
@@ -12,15 +12,16 @@
     <sheet name="Validation" sheetId="7" r:id="rId7"/>
     <sheet name="Protected Input" sheetId="8" r:id="rId8"/>
     <sheet name="Hyperlinks" sheetId="9" r:id="rId9"/>
-    <sheet name="Native Excel Table" sheetId="10" r:id="rId10"/>
-    <sheet name="Grouped Formula Scope" sheetId="11" r:id="rId11"/>
+    <sheet name="Images" sheetId="10" r:id="rId10"/>
+    <sheet name="Native Excel Table" sheetId="11" r:id="rId11"/>
+    <sheet name="Grouped Formula Scope" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
   <si>
     <t>Sparkline Gallery</t>
   </si>
@@ -330,6 +331,21 @@
   </si>
   <si>
     <t>Linked Customer Records</t>
+  </si>
+  <si>
+    <t>Product Image Renderer</t>
+  </si>
+  <si>
+    <t>Photo</t>
+  </si>
+  <si>
+    <t>Product</t>
+  </si>
+  <si>
+    <t>Assembly node kit</t>
+  </si>
+  <si>
+    <t>Retail POS device</t>
   </si>
   <si>
     <t>Region</t>
@@ -703,6 +719,110 @@
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="400050" cy="400050"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1" descr="Assembly node kit"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rIdImage1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="400050" cy="400050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="400050" cy="400050"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 2" descr="Workspace license"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rIdImage2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="400050" cy="400050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>19050</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="400050" cy="400050"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 3" descr="Retail POS device"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rIdImage3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="400050" cy="400050"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="KitchenSinkOrders" displayName="KitchenSinkOrders" ref="A1:G6" totalsRowCount="1" headerRowCount="1">
   <autoFilter ref="A1:G5"/>
@@ -1291,6 +1411,83 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="30"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="29" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>104</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" ht="34.5" customHeight="1">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="D3" s="12">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="4" ht="34.5" customHeight="1">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" s="12">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" ht="34.5" customHeight="1">
+      <c r="A5" s="9"/>
+      <c r="B5" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="D5" s="12">
+        <v>520</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <drawing r:id="rIdDrawing1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
@@ -1438,7 +1635,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="30"/>
@@ -1461,22 +1658,22 @@
         <v>80</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
@@ -1487,7 +1684,7 @@
         <v>12550</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D2" s="12">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="AMER"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
@@ -1518,7 +1715,7 @@
         <v>4996</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D3" s="12">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="AMER"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
@@ -1549,7 +1746,7 @@
         <v>195</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="D4" s="12">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="AMER"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
@@ -1580,7 +1777,7 @@
         <v>11480</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D5" s="12">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="AMER"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
@@ -1605,7 +1802,7 @@
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="19" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B6" s="20">
         <f>SUBTOTAL(101,[Amount])</f>

</xml_diff>

<commit_message>
feat(core): add badge and checkbox renderers
</commit_message>
<xml_diff>
--- a/packages/core/examples/playground.xlsx
+++ b/packages/core/examples/playground.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="121">
   <si>
     <t>Sparkline Gallery</t>
   </si>
@@ -95,6 +95,9 @@
     <t>Account</t>
   </si>
   <si>
+    <t>Tier</t>
+  </si>
+  <si>
     <t>Email</t>
   </si>
   <si>
@@ -114,6 +117,9 @@
   </si>
   <si>
     <t>Fulfilled</t>
+  </si>
+  <si>
+    <t>All Done</t>
   </si>
   <si>
     <t>Notes</t>
@@ -147,6 +153,9 @@
     <t>YES</t>
   </si>
   <si>
+    <t>☐</t>
+  </si>
+  <si>
     <t>Priority shipment
 Requires customs docs</t>
   </si>
@@ -216,6 +225,9 @@
   </si>
   <si>
     <t>Starter seats</t>
+  </si>
+  <si>
+    <t>☑</t>
   </si>
   <si>
     <t>Keep starter discount</t>
@@ -390,7 +402,7 @@
     <numFmt numFmtId="168" formatCode="0%"/>
     <numFmt numFmtId="169" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -409,11 +421,19 @@
       <color rgb="FF1F2937"/>
     </font>
     <font>
+      <b/>
+      <color rgb="FF1D4ED8"/>
+    </font>
+    <font>
       <color rgb="FF166534"/>
     </font>
     <font>
       <b/>
       <color rgb="FF166534"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF0F172A"/>
     </font>
     <font>
       <sz val="12"/>
@@ -427,6 +447,10 @@
     </font>
     <font>
       <b/>
+      <color rgb="FF92400E"/>
+    </font>
+    <font>
+      <b/>
     </font>
     <font>
       <b/>
@@ -437,7 +461,7 @@
       <color rgb="FF0563C1"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -477,6 +501,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDBEAFE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCFCE7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF3C7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -559,7 +595,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -588,6 +624,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -597,40 +636,49 @@
     <xf numFmtId="165" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="9" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="12" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="9" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="12" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="9" fillId="8" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="12" fillId="10" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="168" fontId="0" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -651,10 +699,10 @@
       <alignment horizontal="right" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1422,7 +1470,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -1430,51 +1478,51 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="8" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" ht="34.5" customHeight="1">
       <c r="A3" s="9"/>
       <c r="B3" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="D3" s="12">
+        <v>109</v>
+      </c>
+      <c r="D3" s="13">
         <v>1450</v>
       </c>
     </row>
     <row r="4" ht="34.5" customHeight="1">
       <c r="A4" s="9"/>
       <c r="B4" s="9" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="D4" s="12">
+        <v>54</v>
+      </c>
+      <c r="D4" s="13">
         <v>79</v>
       </c>
     </row>
     <row r="5" ht="34.5" customHeight="1">
       <c r="A5" s="9"/>
       <c r="B5" s="9" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="D5" s="12">
+        <v>110</v>
+      </c>
+      <c r="D5" s="13">
         <v>520</v>
       </c>
     </row>
@@ -1511,119 +1559,119 @@
         <v>23</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2" s="11">
+        <v>39</v>
+      </c>
+      <c r="E2" s="12">
         <v>2</v>
       </c>
-      <c r="F2" s="12">
+      <c r="F2" s="13">
         <v>12550</v>
       </c>
-      <c r="G2" s="16">
+      <c r="G2" s="18">
         <v>45719.395833333336</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="E3" s="11">
+        <v>52</v>
+      </c>
+      <c r="E3" s="12">
         <v>3</v>
       </c>
-      <c r="F3" s="12">
+      <c r="F3" s="13">
         <v>4996</v>
       </c>
-      <c r="G3" s="16">
+      <c r="G3" s="18">
         <v>45723.395833333336</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="E4" s="11">
+        <v>64</v>
+      </c>
+      <c r="E4" s="12">
         <v>1</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="13">
         <v>195</v>
       </c>
-      <c r="G4" s="16">
+      <c r="G4" s="18">
         <v>45728.395833333336</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E5" s="11">
+        <v>72</v>
+      </c>
+      <c r="E5" s="12">
         <v>2</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="13">
         <v>11480</v>
       </c>
-      <c r="G5" s="16">
+      <c r="G5" s="18">
         <v>45734.395833333336</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="F6" s="20">
+      <c r="A6" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="F6" s="24">
         <f>SUBTOTAL(109,[Line Total])</f>
         <v>29221</v>
       </c>
-      <c r="G6" s="24">
+      <c r="G6" s="28">
         <f>SUBTOTAL(104,[Created])</f>
         <v>45734.395833333336</v>
       </c>
@@ -1655,164 +1703,164 @@
         <v>22</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B2" s="12">
+        <v>37</v>
+      </c>
+      <c r="B2" s="13">
         <v>12550</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="D2" s="12">
+        <v>117</v>
+      </c>
+      <c r="D2" s="13">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="AMER"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
         <v>0</v>
       </c>
-      <c r="E2" s="12">
+      <c r="E2" s="13">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="APAC"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
         <v>0</v>
       </c>
-      <c r="F2" s="12">
+      <c r="F2" s="13">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="EMEA"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
         <v>12550</v>
       </c>
-      <c r="G2" s="12">
+      <c r="G2" s="13">
         <f>SUM(grouped_formula_orders[[#This Row],[AMER Amount]],grouped_formula_orders[[#This Row],[APAC Amount]],grouped_formula_orders[[#This Row],[EMEA Amount]])</f>
         <v>12550</v>
       </c>
-      <c r="H2" s="12">
+      <c r="H2" s="13">
         <f>ROUND(AVERAGE(grouped_formula_orders[[#This Row],[AMER Amount]],grouped_formula_orders[[#This Row],[APAC Amount]],grouped_formula_orders[[#This Row],[EMEA Amount]]),2)</f>
         <v>4183.33</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B3" s="12">
+        <v>50</v>
+      </c>
+      <c r="B3" s="13">
         <v>4996</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="D3" s="12">
+        <v>118</v>
+      </c>
+      <c r="D3" s="13">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="AMER"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
         <v>4996</v>
       </c>
-      <c r="E3" s="12">
+      <c r="E3" s="13">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="APAC"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
         <v>0</v>
       </c>
-      <c r="F3" s="12">
+      <c r="F3" s="13">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="EMEA"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
         <v>0</v>
       </c>
-      <c r="G3" s="12">
+      <c r="G3" s="13">
         <f>SUM(grouped_formula_orders[[#This Row],[AMER Amount]],grouped_formula_orders[[#This Row],[APAC Amount]],grouped_formula_orders[[#This Row],[EMEA Amount]])</f>
         <v>4996</v>
       </c>
-      <c r="H3" s="12">
+      <c r="H3" s="13">
         <f>ROUND(AVERAGE(grouped_formula_orders[[#This Row],[AMER Amount]],grouped_formula_orders[[#This Row],[APAC Amount]],grouped_formula_orders[[#This Row],[EMEA Amount]]),2)</f>
         <v>1665.33</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" s="12">
+        <v>62</v>
+      </c>
+      <c r="B4" s="13">
         <v>195</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="D4" s="12">
+        <v>119</v>
+      </c>
+      <c r="D4" s="13">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="AMER"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
         <v>0</v>
       </c>
-      <c r="E4" s="12">
+      <c r="E4" s="13">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="APAC"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
         <v>195</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="13">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="EMEA"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
         <v>0</v>
       </c>
-      <c r="G4" s="12">
+      <c r="G4" s="13">
         <f>SUM(grouped_formula_orders[[#This Row],[AMER Amount]],grouped_formula_orders[[#This Row],[APAC Amount]],grouped_formula_orders[[#This Row],[EMEA Amount]])</f>
         <v>195</v>
       </c>
-      <c r="H4" s="12">
+      <c r="H4" s="13">
         <f>ROUND(AVERAGE(grouped_formula_orders[[#This Row],[AMER Amount]],grouped_formula_orders[[#This Row],[APAC Amount]],grouped_formula_orders[[#This Row],[EMEA Amount]]),2)</f>
         <v>65</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="B5" s="12">
+        <v>71</v>
+      </c>
+      <c r="B5" s="13">
         <v>11480</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="D5" s="12">
+        <v>117</v>
+      </c>
+      <c r="D5" s="13">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="AMER"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
         <v>0</v>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="13">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="APAC"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
         <v>0</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="13">
         <f>IF((grouped_formula_orders[[#This Row],[Region]]="EMEA"),grouped_formula_orders[[#This Row],[Amount]],0)</f>
         <v>11480</v>
       </c>
-      <c r="G5" s="12">
+      <c r="G5" s="13">
         <f>SUM(grouped_formula_orders[[#This Row],[AMER Amount]],grouped_formula_orders[[#This Row],[APAC Amount]],grouped_formula_orders[[#This Row],[EMEA Amount]])</f>
         <v>11480</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="13">
         <f>ROUND(AVERAGE(grouped_formula_orders[[#This Row],[AMER Amount]],grouped_formula_orders[[#This Row],[APAC Amount]],grouped_formula_orders[[#This Row],[EMEA Amount]]),2)</f>
         <v>3826.67</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="19" t="s">
-        <v>116</v>
-      </c>
-      <c r="B6" s="20">
+      <c r="A6" s="23" t="s">
+        <v>120</v>
+      </c>
+      <c r="B6" s="24">
         <f>SUBTOTAL(101,[Amount])</f>
         <v>7305.25</v>
       </c>
-      <c r="G6" s="20">
+      <c r="G6" s="24">
         <f>SUBTOTAL(109,[Regional Total])</f>
         <v>29221</v>
       </c>
-      <c r="H6" s="20">
+      <c r="H6" s="24">
         <f>SUBTOTAL(101,[Regional Avg])</f>
         <v>2435.0825</v>
       </c>
@@ -1826,41 +1874,45 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W24"/>
+  <dimension ref="A1:Y24"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="29" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="5" max="5" width="29" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="7" max="7" width="30" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="10" max="10" width="17" customWidth="1"/>
+    <col min="11" max="11" width="17" customWidth="1"/>
+    <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="13" max="13" width="32" customWidth="1"/>
+    <col min="14" max="14" width="42" customWidth="1"/>
+    <col min="15" max="15" width="27" customWidth="1"/>
+    <col min="18" max="18" width="17" customWidth="1"/>
+    <col min="19" max="19" width="23" customWidth="1"/>
+    <col min="20" max="20" width="23" customWidth="1"/>
+    <col min="21" max="21" width="17" customWidth="1"/>
+    <col min="22" max="22" width="30" customWidth="1"/>
+    <col min="23" max="23" width="13" customWidth="1"/>
+    <col min="24" max="24" width="17" customWidth="1"/>
+    <col min="25" max="25" width="32" customWidth="1"/>
+    <col min="1" max="1" width="17" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
     <col min="5" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1"/>
     <col min="8" max="8" width="17" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
-    <col min="11" max="11" width="32" customWidth="1"/>
-    <col min="12" max="12" width="42" customWidth="1"/>
+    <col min="11" max="11" width="15" customWidth="1"/>
+    <col min="12" max="12" width="32" customWidth="1"/>
     <col min="13" max="13" width="27" customWidth="1"/>
-    <col min="16" max="16" width="17" customWidth="1"/>
-    <col min="17" max="17" width="23" customWidth="1"/>
-    <col min="18" max="18" width="23" customWidth="1"/>
-    <col min="19" max="19" width="17" customWidth="1"/>
-    <col min="20" max="20" width="30" customWidth="1"/>
-    <col min="21" max="21" width="13" customWidth="1"/>
-    <col min="22" max="22" width="17" customWidth="1"/>
-    <col min="23" max="23" width="32" customWidth="1"/>
-    <col min="1" max="1" width="17" customWidth="1"/>
-    <col min="2" max="2" width="23" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="13" customWidth="1"/>
-    <col min="7" max="7" width="17" customWidth="1"/>
-    <col min="8" max="8" width="17" customWidth="1"/>
-    <col min="9" max="9" width="17" customWidth="1"/>
-    <col min="10" max="10" width="32" customWidth="1"/>
-    <col min="11" max="11" width="27" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1879,16 +1931,18 @@
       <c r="K1" s="7"/>
       <c r="L1" s="7"/>
       <c r="M1" s="7"/>
-      <c r="P1" s="7" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="R1" s="7" t="s">
+        <v>79</v>
+      </c>
       <c r="S1" s="7"/>
       <c r="T1" s="7"/>
       <c r="U1" s="7"/>
       <c r="V1" s="7"/>
       <c r="W1" s="7"/>
+      <c r="X1" s="7"/>
+      <c r="Y1" s="7"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="8" t="s">
@@ -1930,362 +1984,398 @@
       <c r="M2" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="N2" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="R2" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="S2" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="R2" s="8" t="s">
+      <c r="T2" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="S2" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="T2" s="8" t="s">
+      <c r="U2" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="U2" s="8" t="s">
+      <c r="V2" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="V2" s="8" t="s">
-        <v>29</v>
-      </c>
       <c r="W2" s="8" t="s">
-        <v>31</v>
+        <v>28</v>
+      </c>
+      <c r="X2" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="Y2" s="8" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>13</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F3" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="11">
+      <c r="F3" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" s="12">
         <v>8</v>
       </c>
-      <c r="H3" s="12">
+      <c r="I3" s="13">
         <v>1450</v>
       </c>
-      <c r="I3" s="13">
+      <c r="J3" s="14">
         <v>11600</v>
       </c>
-      <c r="J3" s="14" t="s">
-        <v>40</v>
-      </c>
       <c r="K3" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="L3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M3" s="16">
+      <c r="L3" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="M3" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="N3" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="O3" s="18">
         <v>45719.395833333336</v>
-      </c>
-      <c r="P3" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q3" s="9" t="s">
-        <v>35</v>
       </c>
       <c r="R3" s="9" t="s">
         <v>36</v>
       </c>
       <c r="S3" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="T3" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="T3" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="U3" s="11">
+      <c r="U3" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="V3" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="W3" s="12">
         <v>8</v>
       </c>
-      <c r="V3" s="13">
+      <c r="X3" s="14">
         <v>11600</v>
       </c>
-      <c r="W3" s="15" t="s">
-        <v>41</v>
+      <c r="Y3" s="17" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="9"/>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="G4" s="11">
+      <c r="D4" s="10"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" s="12">
         <v>1</v>
       </c>
-      <c r="H4" s="12">
+      <c r="I4" s="13">
         <v>950</v>
       </c>
-      <c r="I4" s="17">
+      <c r="J4" s="19">
         <v>950</v>
       </c>
-      <c r="J4" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="K4" s="15"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="16"/>
-      <c r="P4" s="9"/>
-      <c r="Q4" s="9"/>
+      <c r="K4" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="L4" s="16"/>
+      <c r="M4" s="17"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="18"/>
       <c r="R4" s="9"/>
-      <c r="S4" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="T4" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="U4" s="11">
+      <c r="S4" s="9"/>
+      <c r="T4" s="9"/>
+      <c r="U4" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="V4" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="W4" s="12">
         <v>1</v>
       </c>
-      <c r="V4" s="17">
+      <c r="X4" s="19">
         <v>950</v>
       </c>
-      <c r="W4" s="15"/>
+      <c r="Y4" s="17"/>
     </row>
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>14</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="G5" s="11">
+        <v>52</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="H5" s="12">
         <v>24</v>
       </c>
-      <c r="H5" s="12">
+      <c r="I5" s="13">
         <v>79</v>
       </c>
-      <c r="I5" s="13">
+      <c r="J5" s="14">
         <v>1896</v>
       </c>
-      <c r="J5" s="14" t="s">
-        <v>40</v>
-      </c>
       <c r="K5" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="L5" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M5" s="16">
+        <v>42</v>
+      </c>
+      <c r="L5" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="M5" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="O5" s="18">
         <v>45723.395833333336</v>
       </c>
-      <c r="P5" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q5" s="9" t="s">
-        <v>67</v>
-      </c>
       <c r="R5" s="9" t="s">
-        <v>36</v>
+        <v>70</v>
       </c>
       <c r="S5" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="T5" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="U5" s="11">
+        <v>71</v>
+      </c>
+      <c r="T5" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="U5" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="V5" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="W5" s="12">
         <v>14</v>
       </c>
-      <c r="V5" s="13">
+      <c r="X5" s="14">
         <v>7280</v>
       </c>
-      <c r="W5" s="15" t="s">
-        <v>71</v>
+      <c r="Y5" s="17" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="9"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="G6" s="11">
+      <c r="D6" s="21"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="12">
         <v>2</v>
       </c>
-      <c r="H6" s="12">
+      <c r="I6" s="13">
         <v>1250</v>
       </c>
-      <c r="I6" s="13">
+      <c r="J6" s="14">
         <v>2500</v>
       </c>
-      <c r="J6" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="K6" s="15"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="16"/>
-      <c r="P6" s="9"/>
-      <c r="Q6" s="9"/>
+      <c r="K6" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="L6" s="16"/>
+      <c r="M6" s="17"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="18"/>
       <c r="R6" s="9"/>
-      <c r="S6" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="T6" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="U6" s="11">
+      <c r="S6" s="9"/>
+      <c r="T6" s="9"/>
+      <c r="U6" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="V6" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="W6" s="12">
         <v>2</v>
       </c>
-      <c r="V6" s="13">
+      <c r="X6" s="14">
         <v>4200</v>
       </c>
-      <c r="W6" s="15"/>
+      <c r="Y6" s="17"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="G7" s="11">
+      <c r="D7" s="21"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="H7" s="12">
         <v>1</v>
       </c>
-      <c r="H7" s="12">
+      <c r="I7" s="13">
         <v>600</v>
       </c>
-      <c r="I7" s="17">
+      <c r="J7" s="19">
         <v>600</v>
       </c>
-      <c r="J7" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="K7" s="15"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="16"/>
-      <c r="P7" s="19">
+      <c r="K7" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="L7" s="16"/>
+      <c r="M7" s="17"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="18"/>
+      <c r="R7" s="23">
         <v>2</v>
       </c>
-      <c r="U7" s="19">
+      <c r="W7" s="23">
         <v>25</v>
       </c>
-      <c r="V7" s="20">
+      <c r="X7" s="24">
         <v>24030</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>61</v>
+        <v>63</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>15</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="G8" s="11">
+        <v>64</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="H8" s="12">
         <v>5</v>
       </c>
-      <c r="H8" s="12">
+      <c r="I8" s="13">
         <v>39</v>
       </c>
-      <c r="I8" s="13">
+      <c r="J8" s="14">
         <v>195</v>
       </c>
-      <c r="J8" s="14" t="s">
-        <v>40</v>
-      </c>
       <c r="K8" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="L8" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="M8" s="16">
+        <v>42</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="M8" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="N8" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="O8" s="18">
         <v>45728.395833333336</v>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="A9" s="9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B9" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="H9" s="12">
+        <v>14</v>
+      </c>
+      <c r="I9" s="13">
+        <v>520</v>
+      </c>
+      <c r="J9" s="14">
+        <v>7280</v>
+      </c>
+      <c r="K9" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="L9" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="F9" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="G9" s="11">
-        <v>14</v>
-      </c>
-      <c r="H9" s="12">
-        <v>520</v>
-      </c>
-      <c r="I9" s="13">
-        <v>7280</v>
-      </c>
-      <c r="J9" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="K9" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="L9" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="M9" s="16">
+      <c r="M9" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="N9" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="O9" s="18">
         <v>45734.395833333336</v>
       </c>
     </row>
@@ -2293,43 +2383,45 @@
       <c r="A10" s="9"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="G10" s="11">
+      <c r="D10" s="10"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="H10" s="12">
         <v>2</v>
       </c>
-      <c r="H10" s="12">
+      <c r="I10" s="13">
         <v>2100</v>
       </c>
-      <c r="I10" s="13">
+      <c r="J10" s="14">
         <v>4200</v>
       </c>
-      <c r="J10" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="K10" s="15"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="16"/>
+      <c r="K10" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="L10" s="16"/>
+      <c r="M10" s="17"/>
+      <c r="N10" s="9"/>
+      <c r="O10" s="18"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="19">
+      <c r="A11" s="23">
         <v>4</v>
       </c>
-      <c r="G11" s="19">
+      <c r="H11" s="23">
         <v>57</v>
       </c>
-      <c r="I11" s="20">
+      <c r="J11" s="24">
         <v>29221</v>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="7" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -2341,6 +2433,8 @@
       <c r="I14" s="7"/>
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="7"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="8" t="s">
@@ -2353,7 +2447,7 @@
         <v>23</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>26</v>
@@ -2374,41 +2468,53 @@
         <v>31</v>
       </c>
       <c r="K15" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="L15" s="8" t="s">
         <v>33</v>
+      </c>
+      <c r="M15" s="8" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="E16" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="F16" s="11">
+      <c r="D16" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="G16" s="12">
         <v>8</v>
       </c>
-      <c r="G16" s="12">
+      <c r="H16" s="13">
         <v>1450</v>
       </c>
-      <c r="H16" s="13">
+      <c r="I16" s="14">
         <v>11600</v>
       </c>
-      <c r="I16" s="14" t="s">
-        <v>40</v>
-      </c>
       <c r="J16" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="K16" s="16">
+        <v>42</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="L16" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="M16" s="18">
         <v>45719.395833333336</v>
       </c>
     </row>
@@ -2416,59 +2522,67 @@
       <c r="A17" s="9"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>
-      <c r="D17" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E17" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="F17" s="11">
+      <c r="D17" s="10"/>
+      <c r="E17" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17" s="12">
         <v>1</v>
       </c>
-      <c r="G17" s="12">
+      <c r="H17" s="13">
         <v>950</v>
       </c>
-      <c r="H17" s="17">
+      <c r="I17" s="19">
         <v>950</v>
       </c>
-      <c r="I17" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="J17" s="15"/>
+      <c r="J17" s="20" t="s">
+        <v>48</v>
+      </c>
       <c r="K17" s="16"/>
+      <c r="L17" s="17"/>
+      <c r="M17" s="18"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="E18" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="F18" s="11">
+      <c r="D18" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="G18" s="12">
         <v>24</v>
       </c>
-      <c r="G18" s="12">
+      <c r="H18" s="13">
         <v>79</v>
       </c>
-      <c r="H18" s="13">
+      <c r="I18" s="14">
         <v>1896</v>
       </c>
-      <c r="I18" s="14" t="s">
-        <v>40</v>
-      </c>
       <c r="J18" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="K18" s="16">
+        <v>42</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="L18" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="M18" s="18">
         <v>45723.395833333336</v>
       </c>
     </row>
@@ -2476,119 +2590,135 @@
       <c r="A19" s="9"/>
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
-      <c r="D19" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="E19" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="F19" s="11">
+      <c r="D19" s="21"/>
+      <c r="E19" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="G19" s="12">
         <v>2</v>
       </c>
-      <c r="G19" s="12">
+      <c r="H19" s="13">
         <v>1250</v>
       </c>
-      <c r="H19" s="13">
+      <c r="I19" s="14">
         <v>2500</v>
       </c>
-      <c r="I19" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="J19" s="15"/>
+      <c r="J19" s="15" t="s">
+        <v>42</v>
+      </c>
       <c r="K19" s="16"/>
+      <c r="L19" s="17"/>
+      <c r="M19" s="18"/>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="9"/>
       <c r="B20" s="9"/>
       <c r="C20" s="9"/>
-      <c r="D20" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="F20" s="11">
+      <c r="D20" s="21"/>
+      <c r="E20" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G20" s="12">
         <v>1</v>
       </c>
-      <c r="G20" s="12">
+      <c r="H20" s="13">
         <v>600</v>
       </c>
-      <c r="H20" s="17">
+      <c r="I20" s="19">
         <v>600</v>
       </c>
-      <c r="I20" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="J20" s="15"/>
+      <c r="J20" s="20" t="s">
+        <v>48</v>
+      </c>
       <c r="K20" s="16"/>
+      <c r="L20" s="17"/>
+      <c r="M20" s="18"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="E21" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="F21" s="11">
+      <c r="D21" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="G21" s="12">
         <v>5</v>
       </c>
-      <c r="G21" s="12">
+      <c r="H21" s="13">
         <v>39</v>
       </c>
-      <c r="H21" s="13">
+      <c r="I21" s="14">
         <v>195</v>
       </c>
-      <c r="I21" s="14" t="s">
-        <v>40</v>
-      </c>
       <c r="J21" s="15" t="s">
-        <v>64</v>
-      </c>
-      <c r="K21" s="16">
+        <v>42</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="L21" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="M21" s="18">
         <v>45728.395833333336</v>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1">
       <c r="A22" s="9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B22" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="G22" s="12">
+        <v>14</v>
+      </c>
+      <c r="H22" s="13">
+        <v>520</v>
+      </c>
+      <c r="I22" s="14">
+        <v>7280</v>
+      </c>
+      <c r="J22" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="K22" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="C22" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="E22" s="10" t="s">
-        <v>70</v>
-      </c>
-      <c r="F22" s="11">
-        <v>14</v>
-      </c>
-      <c r="G22" s="12">
-        <v>520</v>
-      </c>
-      <c r="H22" s="13">
-        <v>7280</v>
-      </c>
-      <c r="I22" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="J22" s="15" t="s">
-        <v>71</v>
-      </c>
-      <c r="K22" s="16">
+      <c r="L22" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="M22" s="18">
         <v>45734.395833333336</v>
       </c>
     </row>
@@ -2596,114 +2726,130 @@
       <c r="A23" s="9"/>
       <c r="B23" s="9"/>
       <c r="C23" s="9"/>
-      <c r="D23" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="F23" s="11">
+      <c r="D23" s="10"/>
+      <c r="E23" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="G23" s="12">
         <v>2</v>
       </c>
-      <c r="G23" s="12">
+      <c r="H23" s="13">
         <v>2100</v>
       </c>
-      <c r="H23" s="13">
+      <c r="I23" s="14">
         <v>4200</v>
       </c>
-      <c r="I23" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="J23" s="15"/>
+      <c r="J23" s="15" t="s">
+        <v>42</v>
+      </c>
       <c r="K23" s="16"/>
+      <c r="L23" s="17"/>
+      <c r="M23" s="18"/>
     </row>
     <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="19">
+      <c r="A24" s="23">
         <v>4</v>
       </c>
-      <c r="F24" s="19">
+      <c r="G24" s="23">
         <v>57</v>
       </c>
-      <c r="H24" s="20">
+      <c r="I24" s="24">
         <v>29221</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="47">
-    <mergeCell ref="A1:M1"/>
+  <mergeCells count="59">
+    <mergeCell ref="A1:O1"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="M3:M4"/>
+    <mergeCell ref="N3:N4"/>
+    <mergeCell ref="O3:O4"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="B5:B7"/>
     <mergeCell ref="C5:C7"/>
     <mergeCell ref="D5:D7"/>
-    <mergeCell ref="K5:K7"/>
+    <mergeCell ref="E5:E7"/>
     <mergeCell ref="L5:L7"/>
     <mergeCell ref="M5:M7"/>
+    <mergeCell ref="N5:N7"/>
+    <mergeCell ref="O5:O7"/>
     <mergeCell ref="A9:A10"/>
     <mergeCell ref="B9:B10"/>
     <mergeCell ref="C9:C10"/>
     <mergeCell ref="D9:D10"/>
-    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="E9:E10"/>
     <mergeCell ref="L9:L10"/>
     <mergeCell ref="M9:M10"/>
-    <mergeCell ref="P1:W1"/>
-    <mergeCell ref="P3:P4"/>
-    <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="R1:Y1"/>
     <mergeCell ref="R3:R4"/>
-    <mergeCell ref="W3:W4"/>
-    <mergeCell ref="P5:P6"/>
-    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="S3:S4"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="Y3:Y4"/>
     <mergeCell ref="R5:R6"/>
-    <mergeCell ref="W5:W6"/>
-    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="S5:S6"/>
+    <mergeCell ref="T5:T6"/>
+    <mergeCell ref="Y5:Y6"/>
+    <mergeCell ref="A14:M14"/>
     <mergeCell ref="A16:A17"/>
     <mergeCell ref="B16:B17"/>
     <mergeCell ref="C16:C17"/>
-    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="D16:D17"/>
     <mergeCell ref="K16:K17"/>
+    <mergeCell ref="L16:L17"/>
+    <mergeCell ref="M16:M17"/>
     <mergeCell ref="A18:A20"/>
     <mergeCell ref="B18:B20"/>
     <mergeCell ref="C18:C20"/>
-    <mergeCell ref="J18:J20"/>
+    <mergeCell ref="D18:D20"/>
     <mergeCell ref="K18:K20"/>
+    <mergeCell ref="L18:L20"/>
+    <mergeCell ref="M18:M20"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="B22:B23"/>
     <mergeCell ref="C22:C23"/>
-    <mergeCell ref="J22:J23"/>
+    <mergeCell ref="D22:D23"/>
     <mergeCell ref="K22:K23"/>
+    <mergeCell ref="L22:L23"/>
+    <mergeCell ref="M22:M23"/>
   </mergeCells>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:O8"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
     <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="29" customWidth="1"/>
-    <col min="5" max="5" width="17" customWidth="1"/>
-    <col min="6" max="6" width="30" customWidth="1"/>
-    <col min="7" max="7" width="13" customWidth="1"/>
-    <col min="8" max="8" width="17" customWidth="1"/>
+    <col min="4" max="4" width="19" customWidth="1"/>
+    <col min="5" max="5" width="29" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="7" max="7" width="30" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
     <col min="10" max="10" width="17" customWidth="1"/>
-    <col min="11" max="11" width="32" customWidth="1"/>
-    <col min="12" max="12" width="32" customWidth="1"/>
-    <col min="13" max="13" width="27" customWidth="1"/>
+    <col min="11" max="11" width="17" customWidth="1"/>
+    <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="13" max="13" width="32" customWidth="1"/>
+    <col min="14" max="14" width="32" customWidth="1"/>
+    <col min="15" max="15" width="27" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -2717,6 +2863,8 @@
       <c r="K1" s="7"/>
       <c r="L1" s="7"/>
       <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="8" t="s">
@@ -2758,45 +2906,57 @@
       <c r="M2" s="8" t="s">
         <v>33</v>
       </c>
+      <c r="N2" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>13</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F3" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="G3" s="11">
+      <c r="F3" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" s="12">
         <v>8</v>
       </c>
-      <c r="H3" s="12">
+      <c r="I3" s="13">
         <v>1450</v>
       </c>
-      <c r="I3" s="13">
+      <c r="J3" s="14">
         <v>11600</v>
       </c>
-      <c r="J3" s="14" t="s">
-        <v>40</v>
-      </c>
       <c r="K3" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="L3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M3" s="16">
+      <c r="L3" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="M3" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="N3" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="O3" s="18">
         <v>45719.395833333336</v>
       </c>
     </row>
@@ -2804,67 +2964,75 @@
       <c r="A4" s="9"/>
       <c r="B4" s="9"/>
       <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9" t="s">
-        <v>43</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>44</v>
-      </c>
-      <c r="G4" s="11">
+      <c r="D4" s="10"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" s="12">
         <v>1</v>
       </c>
-      <c r="H4" s="12">
+      <c r="I4" s="13">
         <v>950</v>
       </c>
-      <c r="I4" s="17">
+      <c r="J4" s="19">
         <v>950</v>
       </c>
-      <c r="J4" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="K4" s="15"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="16"/>
+      <c r="K4" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="L4" s="16"/>
+      <c r="M4" s="17"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="18"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>14</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="F5" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="G5" s="11">
+        <v>52</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="H5" s="12">
         <v>24</v>
       </c>
-      <c r="H5" s="12">
+      <c r="I5" s="13">
         <v>79</v>
       </c>
-      <c r="I5" s="13">
+      <c r="J5" s="14">
         <v>1896</v>
       </c>
-      <c r="J5" s="14" t="s">
-        <v>40</v>
-      </c>
       <c r="K5" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="L5" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="M5" s="16">
+        <v>42</v>
+      </c>
+      <c r="L5" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="M5" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="O5" s="18">
         <v>45723.395833333336</v>
       </c>
     </row>
@@ -2872,84 +3040,92 @@
       <c r="A6" s="9"/>
       <c r="B6" s="9"/>
       <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="G6" s="11">
+      <c r="D6" s="21"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="H6" s="12">
         <v>2</v>
       </c>
-      <c r="H6" s="12">
+      <c r="I6" s="13">
         <v>1250</v>
       </c>
-      <c r="I6" s="13">
+      <c r="J6" s="14">
         <v>2500</v>
       </c>
-      <c r="J6" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="K6" s="15"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="16"/>
+      <c r="K6" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="L6" s="16"/>
+      <c r="M6" s="17"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="18"/>
     </row>
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="9"/>
       <c r="B7" s="9"/>
       <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="G7" s="11">
+      <c r="D7" s="21"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="H7" s="12">
         <v>1</v>
       </c>
-      <c r="H7" s="12">
+      <c r="I7" s="13">
         <v>600</v>
       </c>
-      <c r="I7" s="17">
+      <c r="J7" s="19">
         <v>600</v>
       </c>
-      <c r="J7" s="18" t="s">
-        <v>45</v>
-      </c>
-      <c r="K7" s="15"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="16"/>
+      <c r="K7" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="L7" s="16"/>
+      <c r="M7" s="17"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="18"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="19">
+      <c r="A8" s="23">
         <v>2</v>
       </c>
-      <c r="G8" s="19">
+      <c r="H8" s="23">
         <v>36</v>
       </c>
-      <c r="I8" s="20">
+      <c r="J8" s="24">
         <v>17546</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="A1:M1"/>
+  <mergeCells count="19">
+    <mergeCell ref="A1:O1"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="D3:D4"/>
-    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="M3:M4"/>
+    <mergeCell ref="N3:N4"/>
+    <mergeCell ref="O3:O4"/>
     <mergeCell ref="A5:A7"/>
     <mergeCell ref="B5:B7"/>
     <mergeCell ref="C5:C7"/>
     <mergeCell ref="D5:D7"/>
-    <mergeCell ref="K5:K7"/>
+    <mergeCell ref="E5:E7"/>
     <mergeCell ref="L5:L7"/>
     <mergeCell ref="M5:M7"/>
+    <mergeCell ref="N5:N7"/>
+    <mergeCell ref="O5:O7"/>
   </mergeCells>
 </worksheet>
 </file>
@@ -2970,7 +3146,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -2990,112 +3166,112 @@
         <v>23</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>41</v>
+        <v>39</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>44</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="G3" s="16">
+        <v>45</v>
+      </c>
+      <c r="G3" s="18">
         <v>45719.395833333336</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="E4" s="15" t="s">
         <v>52</v>
       </c>
+      <c r="E4" s="17" t="s">
+        <v>55</v>
+      </c>
       <c r="F4" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="G4" s="16">
+        <v>56</v>
+      </c>
+      <c r="G4" s="18">
         <v>45723.395833333336</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>61</v>
-      </c>
-      <c r="E5" s="15" t="s">
         <v>64</v>
       </c>
+      <c r="E5" s="17" t="s">
+        <v>68</v>
+      </c>
       <c r="F5" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="G5" s="16">
+        <v>69</v>
+      </c>
+      <c r="G5" s="18">
         <v>45728.395833333336</v>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>75</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="G6" s="16">
+        <v>76</v>
+      </c>
+      <c r="G6" s="18">
         <v>45734.395833333336</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="19">
+      <c r="A7" s="23">
         <v>4</v>
       </c>
     </row>
@@ -3121,7 +3297,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -3133,115 +3309,115 @@
         <v>22</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3" s="12">
+        <v>37</v>
+      </c>
+      <c r="B3" s="13">
         <v>12550</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="12">
         <v>2</v>
       </c>
-      <c r="D3" s="21">
+      <c r="D3" s="25">
         <v>0.5</v>
       </c>
-      <c r="E3" s="16">
+      <c r="E3" s="18">
         <v>45719.395833333336</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="12">
+        <v>50</v>
+      </c>
+      <c r="B4" s="13">
         <v>4996</v>
       </c>
-      <c r="C4" s="11">
+      <c r="C4" s="12">
         <v>3</v>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="25">
         <v>0.6666666666666666</v>
       </c>
-      <c r="E4" s="16">
+      <c r="E4" s="18">
         <v>45723.395833333336</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" s="12">
+        <v>62</v>
+      </c>
+      <c r="B5" s="13">
         <v>195</v>
       </c>
-      <c r="C5" s="11">
+      <c r="C5" s="12">
         <v>1</v>
       </c>
-      <c r="D5" s="21">
+      <c r="D5" s="25">
         <v>1</v>
       </c>
-      <c r="E5" s="16">
+      <c r="E5" s="18">
         <v>45728.395833333336</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="12">
+        <v>71</v>
+      </c>
+      <c r="B6" s="13">
         <v>11480</v>
       </c>
-      <c r="C6" s="11">
+      <c r="C6" s="12">
         <v>2</v>
       </c>
-      <c r="D6" s="21">
+      <c r="D6" s="25">
         <v>1</v>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="18">
         <v>45734.395833333336</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="19" t="s">
-        <v>83</v>
-      </c>
-      <c r="B7" s="20">
+      <c r="A7" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" s="24">
         <f>ROUND(SUM(B3:B6),2)</f>
       </c>
-      <c r="C7" s="22">
+      <c r="C7" s="26">
         <f>SUM(C3:C6)</f>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="27">
         <f>ROUND(AVERAGE(D3:D6),4)</f>
       </c>
-      <c r="E7" s="19"/>
+      <c r="E7" s="23"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="19" t="s">
-        <v>84</v>
-      </c>
-      <c r="B8" s="20">
+      <c r="A8" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" s="24">
         <f>ROUND(AVERAGE(B3:B6),2)</f>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="26">
         <f>AVERAGE(C3:C6)</f>
       </c>
-      <c r="D8" s="23">
+      <c r="D8" s="27">
         <f>MAX(MAX(D3:D6),0)</f>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="28">
         <f>MAX(MAX(E3:E6),0)</f>
       </c>
     </row>
@@ -3297,7 +3473,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -3314,25 +3490,25 @@
         <v>22</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="E2" s="8" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="I2" s="8" t="s">
         <v>3</v>
@@ -3343,27 +3519,27 @@
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3" s="11">
+        <v>37</v>
+      </c>
+      <c r="B3" s="12">
         <v>9</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3" s="13">
         <v>1200</v>
       </c>
-      <c r="D3" s="25">
+      <c r="D3" s="29">
         <v>0.18</v>
       </c>
-      <c r="E3" s="11">
+      <c r="E3" s="12">
         <v>8</v>
       </c>
-      <c r="F3" s="12">
+      <c r="F3" s="13">
         <f>ROUND((B3*C3),2)</f>
       </c>
-      <c r="G3" s="21">
+      <c r="G3" s="25">
         <f>ROUND(IF((B3&lt;&gt;0),(E3/B3),0),4)</f>
       </c>
-      <c r="H3" s="12">
+      <c r="H3" s="13">
         <f>ROUND((F3*(1-D3)),2)</f>
       </c>
       <c r="I3" s="9">
@@ -3375,27 +3551,27 @@
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="11">
+        <v>50</v>
+      </c>
+      <c r="B4" s="12">
         <v>27</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="13">
         <v>643</v>
       </c>
-      <c r="D4" s="25">
+      <c r="D4" s="29">
         <v>0.1</v>
       </c>
-      <c r="E4" s="11">
+      <c r="E4" s="12">
         <v>26</v>
       </c>
-      <c r="F4" s="12">
+      <c r="F4" s="13">
         <f>ROUND((B4*C4),2)</f>
       </c>
-      <c r="G4" s="21">
+      <c r="G4" s="25">
         <f>ROUND(IF((B4&lt;&gt;0),(E4/B4),0),4)</f>
       </c>
-      <c r="H4" s="12">
+      <c r="H4" s="13">
         <f>ROUND((F4*(1-D4)),2)</f>
       </c>
       <c r="I4" s="9">
@@ -3407,27 +3583,27 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" s="11">
+        <v>62</v>
+      </c>
+      <c r="B5" s="12">
         <v>5</v>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="13">
         <v>39</v>
       </c>
-      <c r="D5" s="25">
+      <c r="D5" s="29">
         <v>0.03</v>
       </c>
-      <c r="E5" s="11">
+      <c r="E5" s="12">
         <v>5</v>
       </c>
-      <c r="F5" s="12">
+      <c r="F5" s="13">
         <f>ROUND((B5*C5),2)</f>
       </c>
-      <c r="G5" s="21">
+      <c r="G5" s="25">
         <f>ROUND(IF((B5&lt;&gt;0),(E5/B5),0),4)</f>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="13">
         <f>ROUND((F5*(1-D5)),2)</f>
       </c>
       <c r="I5" s="9">
@@ -3439,27 +3615,27 @@
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="11">
+        <v>71</v>
+      </c>
+      <c r="B6" s="12">
         <v>16</v>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="13">
         <v>1310</v>
       </c>
-      <c r="D6" s="25">
+      <c r="D6" s="29">
         <v>0.18</v>
       </c>
-      <c r="E6" s="11">
+      <c r="E6" s="12">
         <v>16</v>
       </c>
-      <c r="F6" s="12">
+      <c r="F6" s="13">
         <f>ROUND((B6*C6),2)</f>
       </c>
-      <c r="G6" s="21">
+      <c r="G6" s="25">
         <f>ROUND(IF((B6&lt;&gt;0),(E6/B6),0),4)</f>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="13">
         <f>ROUND((F6*(1-D6)),2)</f>
       </c>
       <c r="I6" s="9">
@@ -3470,10 +3646,10 @@
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="F7" s="20">
+      <c r="F7" s="24">
         <f>ROUND(SUM(F3:F6),2)</f>
       </c>
-      <c r="H7" s="20">
+      <c r="H7" s="24">
         <f>ROUND(SUM(H3:H6),2)</f>
       </c>
     </row>
@@ -3513,7 +3689,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -3521,81 +3697,81 @@
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="8" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="C3" s="12">
+        <v>99</v>
+      </c>
+      <c r="C3" s="13">
         <v>12550</v>
       </c>
-      <c r="D3" s="26">
+      <c r="D3" s="30">
         <v>45719.395833333336</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="9" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="C4" s="12">
+        <v>100</v>
+      </c>
+      <c r="C4" s="13">
         <v>4996</v>
       </c>
-      <c r="D4" s="26">
+      <c r="D4" s="30">
         <v>45723.395833333336</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="C5" s="12">
+        <v>101</v>
+      </c>
+      <c r="C5" s="13">
         <v>195</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="30">
         <v>45728.395833333336</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="9" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="C6" s="12">
+        <v>99</v>
+      </c>
+      <c r="C6" s="13">
         <v>11480</v>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="30">
         <v>45734.395833333336</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="C7" s="19" t="s">
-        <v>83</v>
+      <c r="C7" s="23" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="C8" s="20">
+      <c r="C8" s="24">
         <f>SUM(C3:C6)</f>
       </c>
     </row>
@@ -3630,63 +3806,63 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="8" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="27" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3" s="28">
+      <c r="A3" s="31" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" s="32">
         <v>12550</v>
       </c>
-      <c r="C3" s="29">
+      <c r="C3" s="33">
         <f>ROUND((B3*0.9),0)</f>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="28">
+      <c r="A4" s="31" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" s="32">
         <v>4996</v>
       </c>
-      <c r="C4" s="29">
+      <c r="C4" s="33">
         <f>ROUND((B4*0.9),0)</f>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" s="28">
+      <c r="A5" s="31" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="32">
         <v>195</v>
       </c>
-      <c r="C5" s="29">
+      <c r="C5" s="33">
         <f>ROUND((B5*0.9),0)</f>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="27" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="28">
+      <c r="A6" s="31" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="32">
         <v>11480</v>
       </c>
-      <c r="C6" s="29">
+      <c r="C6" s="33">
         <f>ROUND((B6*0.9),0)</f>
       </c>
     </row>
@@ -3715,7 +3891,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="7" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B1" s="7"/>
     </row>
@@ -3724,39 +3900,39 @@
         <v>22</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3" s="31" t="s">
+      <c r="A3" s="34" t="s">
         <v>37</v>
+      </c>
+      <c r="B3" s="35" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="31" t="s">
-        <v>49</v>
+        <v>50</v>
+      </c>
+      <c r="B4" s="35" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="30" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>61</v>
+      <c r="A5" s="34" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="35" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="B6" s="31" t="s">
-        <v>68</v>
+        <v>71</v>
+      </c>
+      <c r="B6" s="35" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>